<commit_message>
chore(pipeline): refresh slates, grades, and shadow tickets for May 17-19
Update combined tickets, mobile grade artifacts, shadow_tickets_latest.json, sport caches, and daily audit reports from recent pipeline and grader runs.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/ui_runner/templates/graded_analysis_tabs_2026-05-18.xlsx
+++ b/ui_runner/templates/graded_analysis_tabs_2026-05-18.xlsx
@@ -471,16 +471,16 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E2" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F2" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G2" t="n">
-        <v>55.9</v>
+        <v>60</v>
       </c>
     </row>
     <row r="3">
@@ -674,16 +674,16 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="E9" t="n">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F9" t="n">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="G9" t="n">
-        <v>61.2</v>
+        <v>62.1</v>
       </c>
     </row>
     <row r="10">
@@ -732,16 +732,16 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="E11" t="n">
         <v>211</v>
       </c>
       <c r="F11" t="n">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="G11" t="n">
-        <v>60.8</v>
+        <v>61</v>
       </c>
     </row>
     <row r="12">
@@ -819,16 +819,16 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="E14" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F14" t="n">
         <v>149</v>
       </c>
       <c r="G14" t="n">
-        <v>25.1</v>
+        <v>25.5</v>
       </c>
     </row>
     <row r="15">
@@ -848,16 +848,16 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="E15" t="n">
         <v>33</v>
       </c>
       <c r="F15" t="n">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="G15" t="n">
-        <v>13.1</v>
+        <v>13.2</v>
       </c>
     </row>
     <row r="16">
@@ -877,16 +877,16 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E16" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="F16" t="n">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G16" t="n">
-        <v>17.1</v>
+        <v>19.5</v>
       </c>
     </row>
     <row r="17">
@@ -906,13 +906,13 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>2279</v>
+        <v>2276</v>
       </c>
       <c r="E17" t="n">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="F17" t="n">
-        <v>1738</v>
+        <v>1736</v>
       </c>
       <c r="G17" t="n">
         <v>23.7</v>
@@ -1142,19 +1142,19 @@
         <v>15</v>
       </c>
       <c r="N2" t="n">
+        <v>61.5</v>
+      </c>
+      <c r="O2" t="n">
+        <v>13</v>
+      </c>
+      <c r="P2" t="n">
         <v>50</v>
       </c>
-      <c r="O2" t="n">
-        <v>12</v>
-      </c>
-      <c r="P2" t="n">
-        <v>51.1</v>
-      </c>
       <c r="Q2" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="R2" t="n">
-        <v>76.90000000000001</v>
+        <v>84.59999999999999</v>
       </c>
       <c r="S2" t="n">
         <v>13</v>
@@ -1196,7 +1196,7 @@
         <v>5</v>
       </c>
       <c r="AF2" t="n">
-        <v>51.2</v>
+        <v>53.7</v>
       </c>
       <c r="AG2" t="n">
         <v>41</v>
@@ -1215,10 +1215,10 @@
         <v>79</v>
       </c>
       <c r="D3" t="n">
-        <v>52.2</v>
+        <v>53</v>
       </c>
       <c r="E3" t="n">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F3" t="n">
         <v>54.7</v>
@@ -1233,34 +1233,34 @@
         <v>33</v>
       </c>
       <c r="J3" t="n">
-        <v>11.1</v>
+        <v>20</v>
       </c>
       <c r="K3" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="L3" t="n">
-        <v>3</v>
+        <v>3.1</v>
       </c>
       <c r="M3" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="N3" t="n">
-        <v>20</v>
+        <v>23.1</v>
       </c>
       <c r="O3" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="P3" t="n">
-        <v>35.1</v>
+        <v>36</v>
       </c>
       <c r="Q3" t="n">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="R3" t="n">
-        <v>33.3</v>
+        <v>38.5</v>
       </c>
       <c r="S3" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="U3" t="n">
         <v>0</v>
@@ -1290,10 +1290,10 @@
         <v>5</v>
       </c>
       <c r="AF3" t="n">
-        <v>69.09999999999999</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="AG3" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="4">
@@ -1483,10 +1483,10 @@
         <v>571</v>
       </c>
       <c r="D7" t="n">
-        <v>60.8</v>
+        <v>61</v>
       </c>
       <c r="E7" t="n">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="F7" t="n">
         <v>68</v>
@@ -1501,34 +1501,34 @@
         <v>122</v>
       </c>
       <c r="J7" t="n">
-        <v>25.1</v>
+        <v>25.5</v>
       </c>
       <c r="K7" t="n">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="L7" t="n">
-        <v>13.1</v>
+        <v>13.2</v>
       </c>
       <c r="M7" t="n">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="N7" t="n">
-        <v>17.1</v>
+        <v>19.5</v>
       </c>
       <c r="O7" t="n">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="P7" t="n">
         <v>23.7</v>
       </c>
       <c r="Q7" t="n">
-        <v>2279</v>
+        <v>2276</v>
       </c>
       <c r="R7" t="n">
-        <v>55.9</v>
+        <v>60</v>
       </c>
       <c r="S7" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="T7" t="n">
         <v>41.2</v>
@@ -1567,10 +1567,10 @@
         <v>31</v>
       </c>
       <c r="AF7" t="n">
-        <v>61.2</v>
+        <v>62.1</v>
       </c>
       <c r="AG7" t="n">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily slate 2026-05-20 [auto]
</commit_message>
<xml_diff>
--- a/ui_runner/templates/graded_analysis_tabs_2026-05-18.xlsx
+++ b/ui_runner/templates/graded_analysis_tabs_2026-05-18.xlsx
@@ -558,16 +558,16 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E5" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F5" t="n">
         <v>26</v>
       </c>
       <c r="G5" t="n">
-        <v>33.3</v>
+        <v>36.6</v>
       </c>
     </row>
     <row r="6">
@@ -587,16 +587,16 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E6" t="n">
         <v>20</v>
       </c>
       <c r="F6" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G6" t="n">
-        <v>54.1</v>
+        <v>52.6</v>
       </c>
     </row>
     <row r="7">
@@ -616,16 +616,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E7" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F7" t="n">
         <v>10</v>
       </c>
       <c r="G7" t="n">
-        <v>67.7</v>
+        <v>68.8</v>
       </c>
     </row>
     <row r="8">
@@ -645,16 +645,16 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>728</v>
+        <v>730</v>
       </c>
       <c r="E8" t="n">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="F8" t="n">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="G8" t="n">
-        <v>32.1</v>
+        <v>32.2</v>
       </c>
     </row>
     <row r="9">
@@ -674,16 +674,16 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="E9" t="n">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="F9" t="n">
         <v>74</v>
       </c>
       <c r="G9" t="n">
-        <v>62.1</v>
+        <v>62.8</v>
       </c>
     </row>
     <row r="10">
@@ -703,16 +703,16 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>571</v>
+        <v>594</v>
       </c>
       <c r="E10" t="n">
-        <v>365</v>
+        <v>375</v>
       </c>
       <c r="F10" t="n">
-        <v>206</v>
+        <v>219</v>
       </c>
       <c r="G10" t="n">
-        <v>63.9</v>
+        <v>63.1</v>
       </c>
     </row>
     <row r="11">
@@ -732,16 +732,16 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>346</v>
+        <v>354</v>
       </c>
       <c r="E11" t="n">
-        <v>211</v>
+        <v>219</v>
       </c>
       <c r="F11" t="n">
         <v>135</v>
       </c>
       <c r="G11" t="n">
-        <v>61</v>
+        <v>61.9</v>
       </c>
     </row>
     <row r="12">
@@ -761,16 +761,16 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="E12" t="n">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="F12" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="G12" t="n">
-        <v>68</v>
+        <v>68.2</v>
       </c>
     </row>
     <row r="13">
@@ -790,16 +790,16 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E13" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F13" t="n">
         <v>41</v>
       </c>
       <c r="G13" t="n">
-        <v>66.40000000000001</v>
+        <v>66.7</v>
       </c>
     </row>
     <row r="14">
@@ -819,16 +819,16 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>200</v>
+        <v>207</v>
       </c>
       <c r="E14" t="n">
         <v>51</v>
       </c>
       <c r="F14" t="n">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="G14" t="n">
-        <v>25.5</v>
+        <v>24.6</v>
       </c>
     </row>
     <row r="15">
@@ -848,16 +848,16 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="E15" t="n">
         <v>33</v>
       </c>
       <c r="F15" t="n">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="G15" t="n">
-        <v>13.2</v>
+        <v>13</v>
       </c>
     </row>
     <row r="16">
@@ -877,16 +877,16 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E16" t="n">
         <v>22</v>
       </c>
       <c r="F16" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="G16" t="n">
-        <v>19.5</v>
+        <v>19.3</v>
       </c>
     </row>
     <row r="17">
@@ -906,16 +906,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>2276</v>
+        <v>2390</v>
       </c>
       <c r="E17" t="n">
-        <v>540</v>
+        <v>554</v>
       </c>
       <c r="F17" t="n">
-        <v>1736</v>
+        <v>1836</v>
       </c>
       <c r="G17" t="n">
-        <v>23.7</v>
+        <v>23.2</v>
       </c>
     </row>
   </sheetData>
@@ -1477,52 +1477,52 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>63.9</v>
+        <v>63.1</v>
       </c>
       <c r="C7" t="n">
-        <v>571</v>
+        <v>594</v>
       </c>
       <c r="D7" t="n">
-        <v>61</v>
+        <v>61.9</v>
       </c>
       <c r="E7" t="n">
-        <v>346</v>
+        <v>354</v>
       </c>
       <c r="F7" t="n">
-        <v>68</v>
+        <v>68.2</v>
       </c>
       <c r="G7" t="n">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="H7" t="n">
-        <v>66.40000000000001</v>
+        <v>66.7</v>
       </c>
       <c r="I7" t="n">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="J7" t="n">
-        <v>25.5</v>
+        <v>24.6</v>
       </c>
       <c r="K7" t="n">
-        <v>200</v>
+        <v>207</v>
       </c>
       <c r="L7" t="n">
-        <v>13.2</v>
+        <v>13</v>
       </c>
       <c r="M7" t="n">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="N7" t="n">
-        <v>19.5</v>
+        <v>19.3</v>
       </c>
       <c r="O7" t="n">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="P7" t="n">
-        <v>23.7</v>
+        <v>23.2</v>
       </c>
       <c r="Q7" t="n">
-        <v>2276</v>
+        <v>2390</v>
       </c>
       <c r="R7" t="n">
         <v>60</v>
@@ -1537,16 +1537,16 @@
         <v>17</v>
       </c>
       <c r="V7" t="n">
-        <v>54.1</v>
+        <v>52.6</v>
       </c>
       <c r="W7" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="X7" t="n">
-        <v>32.1</v>
+        <v>32.2</v>
       </c>
       <c r="Y7" t="n">
-        <v>728</v>
+        <v>730</v>
       </c>
       <c r="Z7" t="n">
         <v>65.09999999999999</v>
@@ -1555,22 +1555,22 @@
         <v>43</v>
       </c>
       <c r="AB7" t="n">
-        <v>33.3</v>
+        <v>36.6</v>
       </c>
       <c r="AC7" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="AD7" t="n">
-        <v>67.7</v>
+        <v>68.8</v>
       </c>
       <c r="AE7" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="AF7" t="n">
-        <v>62.1</v>
+        <v>62.8</v>
       </c>
       <c r="AG7" t="n">
-        <v>195</v>
+        <v>199</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily slate 2026-06-03 [auto]
</commit_message>
<xml_diff>
--- a/ui_runner/templates/graded_analysis_tabs_2026-05-18.xlsx
+++ b/ui_runner/templates/graded_analysis_tabs_2026-05-18.xlsx
@@ -471,16 +471,16 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>49</v>
+        <v>72</v>
       </c>
       <c r="E2" t="n">
-        <v>29</v>
+        <v>46</v>
       </c>
       <c r="F2" t="n">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="G2" t="n">
-        <v>59.2</v>
+        <v>63.9</v>
       </c>
     </row>
     <row r="3">
@@ -529,16 +529,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="E4" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F4" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="G4" t="n">
-        <v>43.5</v>
+        <v>42.9</v>
       </c>
     </row>
     <row r="5">
@@ -558,16 +558,16 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>44</v>
+        <v>56</v>
       </c>
       <c r="E5" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="F5" t="n">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="G5" t="n">
-        <v>36.4</v>
+        <v>41.1</v>
       </c>
     </row>
     <row r="6">
@@ -616,16 +616,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="E7" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="F7" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G7" t="n">
-        <v>66.7</v>
+        <v>65</v>
       </c>
     </row>
     <row r="8">
@@ -645,16 +645,16 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>721</v>
+        <v>675</v>
       </c>
       <c r="E8" t="n">
-        <v>230</v>
+        <v>205</v>
       </c>
       <c r="F8" t="n">
-        <v>491</v>
+        <v>470</v>
       </c>
       <c r="G8" t="n">
-        <v>31.9</v>
+        <v>30.4</v>
       </c>
     </row>
     <row r="9">
@@ -674,16 +674,16 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>209</v>
+        <v>195</v>
       </c>
       <c r="E9" t="n">
-        <v>132</v>
+        <v>123</v>
       </c>
       <c r="F9" t="n">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="G9" t="n">
-        <v>63.2</v>
+        <v>63.1</v>
       </c>
     </row>
     <row r="10">
@@ -706,13 +706,13 @@
         <v>594</v>
       </c>
       <c r="E10" t="n">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="F10" t="n">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="G10" t="n">
-        <v>63.6</v>
+        <v>63.3</v>
       </c>
     </row>
     <row r="11">
@@ -790,16 +790,16 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>305</v>
+        <v>124</v>
       </c>
       <c r="E13" t="n">
-        <v>165</v>
+        <v>82</v>
       </c>
       <c r="F13" t="n">
-        <v>140</v>
+        <v>42</v>
       </c>
       <c r="G13" t="n">
-        <v>54.1</v>
+        <v>66.09999999999999</v>
       </c>
     </row>
     <row r="14">
@@ -906,16 +906,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>2531</v>
+        <v>2291</v>
       </c>
       <c r="E17" t="n">
-        <v>522</v>
+        <v>514</v>
       </c>
       <c r="F17" t="n">
-        <v>2009</v>
+        <v>1777</v>
       </c>
       <c r="G17" t="n">
-        <v>20.6</v>
+        <v>22.4</v>
       </c>
     </row>
   </sheetData>
@@ -1154,16 +1154,16 @@
         <v>4</v>
       </c>
       <c r="R2" t="n">
-        <v>84.59999999999999</v>
+        <v>82.09999999999999</v>
       </c>
       <c r="S2" t="n">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="T2" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="U2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="V2" t="n">
         <v>0</v>
@@ -1172,22 +1172,22 @@
         <v>1</v>
       </c>
       <c r="X2" t="n">
-        <v>51.1</v>
+        <v>48.7</v>
       </c>
       <c r="Y2" t="n">
-        <v>174</v>
+        <v>158</v>
       </c>
       <c r="Z2" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="AA2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AB2" t="n">
-        <v>7.1</v>
+        <v>21.1</v>
       </c>
       <c r="AC2" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="AD2" t="n">
         <v>25</v>
@@ -1196,10 +1196,10 @@
         <v>4</v>
       </c>
       <c r="AF2" t="n">
-        <v>52.4</v>
+        <v>50</v>
       </c>
       <c r="AG2" t="n">
-        <v>42</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3">
@@ -1327,37 +1327,43 @@
         <v>0</v>
       </c>
       <c r="R4" t="n">
-        <v>66.7</v>
+        <v>63.6</v>
       </c>
       <c r="S4" t="n">
+        <v>11</v>
+      </c>
+      <c r="T4" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="U4" t="n">
         <v>3</v>
       </c>
-      <c r="U4" t="n">
-        <v>0</v>
-      </c>
       <c r="W4" t="n">
         <v>0</v>
       </c>
       <c r="X4" t="n">
-        <v>24.6</v>
+        <v>22.6</v>
       </c>
       <c r="Y4" t="n">
-        <v>126</v>
+        <v>115</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>100</v>
       </c>
       <c r="AA4" t="n">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="AB4" t="n">
+        <v>57.1</v>
       </c>
       <c r="AC4" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="AE4" t="n">
         <v>0</v>
       </c>
-      <c r="AF4" t="n">
-        <v>66.7</v>
-      </c>
       <c r="AG4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -1477,7 +1483,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>63.6</v>
+        <v>63.3</v>
       </c>
       <c r="C7" t="n">
         <v>594</v>
@@ -1495,10 +1501,10 @@
         <v>201</v>
       </c>
       <c r="H7" t="n">
-        <v>54.1</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="I7" t="n">
-        <v>305</v>
+        <v>124</v>
       </c>
       <c r="J7" t="n">
         <v>23.7</v>
@@ -1519,22 +1525,22 @@
         <v>105</v>
       </c>
       <c r="P7" t="n">
-        <v>20.6</v>
+        <v>22.4</v>
       </c>
       <c r="Q7" t="n">
-        <v>2531</v>
+        <v>2291</v>
       </c>
       <c r="R7" t="n">
-        <v>59.2</v>
+        <v>63.9</v>
       </c>
       <c r="S7" t="n">
-        <v>49</v>
+        <v>72</v>
       </c>
       <c r="T7" t="n">
-        <v>43.5</v>
+        <v>42.9</v>
       </c>
       <c r="U7" t="n">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="V7" t="n">
         <v>52.1</v>
@@ -1543,10 +1549,10 @@
         <v>48</v>
       </c>
       <c r="X7" t="n">
-        <v>31.9</v>
+        <v>30.4</v>
       </c>
       <c r="Y7" t="n">
-        <v>721</v>
+        <v>675</v>
       </c>
       <c r="Z7" t="n">
         <v>65.09999999999999</v>
@@ -1555,22 +1561,22 @@
         <v>43</v>
       </c>
       <c r="AB7" t="n">
-        <v>36.4</v>
+        <v>41.1</v>
       </c>
       <c r="AC7" t="n">
-        <v>44</v>
+        <v>56</v>
       </c>
       <c r="AD7" t="n">
-        <v>66.7</v>
+        <v>65</v>
       </c>
       <c r="AE7" t="n">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="AF7" t="n">
-        <v>63.2</v>
+        <v>63.1</v>
       </c>
       <c r="AG7" t="n">
-        <v>209</v>
+        <v>195</v>
       </c>
     </row>
   </sheetData>

</xml_diff>